<commit_message>
Import existing merchant history with reviewed balances and fix installer checks
</commit_message>
<xml_diff>
--- a/docs/qa/mcube-cash.xlsx
+++ b/docs/qa/mcube-cash.xlsx
@@ -28,7 +28,7 @@
     <t>Reference</t>
   </si>
   <si>
-    <t>REPORT-2026-10-13-000b8369</t>
+    <t>REPORT-2026-10-13-b7f855f3</t>
   </si>
   <si>
     <t>Prepared by</t>
@@ -40,7 +40,7 @@
     <t>Generated</t>
   </si>
   <si>
-    <t>13 Oct 2026, 15:46</t>
+    <t>13 Oct 2026, 22:41</t>
   </si>
   <si>
     <t>A. Opening Cash</t>

</xml_diff>

<commit_message>
Harden notification dispatch and review duplicate imported payments
</commit_message>
<xml_diff>
--- a/docs/qa/mcube-cash.xlsx
+++ b/docs/qa/mcube-cash.xlsx
@@ -28,7 +28,7 @@
     <t>Reference</t>
   </si>
   <si>
-    <t>REPORT-2026-10-13-b7f855f3</t>
+    <t>REPORT-2026-10-13-7d240d74</t>
   </si>
   <si>
     <t>Prepared by</t>
@@ -40,7 +40,7 @@
     <t>Generated</t>
   </si>
   <si>
-    <t>13 Oct 2026, 22:41</t>
+    <t>13 Oct 2026, 23:28</t>
   </si>
   <si>
     <t>A. Opening Cash</t>

</xml_diff>

<commit_message>
Join historical merchant and payment sheets and retain references in shared history
</commit_message>
<xml_diff>
--- a/docs/qa/mcube-cash.xlsx
+++ b/docs/qa/mcube-cash.xlsx
@@ -28,7 +28,7 @@
     <t>Reference</t>
   </si>
   <si>
-    <t>REPORT-2026-10-13-7d240d74</t>
+    <t>REPORT-2026-10-13-4e012bf6</t>
   </si>
   <si>
     <t>Prepared by</t>
@@ -40,7 +40,7 @@
     <t>Generated</t>
   </si>
   <si>
-    <t>13 Oct 2026, 23:28</t>
+    <t>13 Oct 2026, 23:44</t>
   </si>
   <si>
     <t>A. Opening Cash</t>

</xml_diff>